<commit_message>
Add new intake 1234
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,30 +429,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-17062</v>
+        <v>1234</v>
       </c>
       <c r="B2" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>qwer2</v>
       </c>
       <c r="C2" t="str">
-        <v>Invite to JRM</v>
+        <v>qwer2</v>
       </c>
       <c r="D2" t="str">
-        <v>FLCM</v>
+        <v>flcm</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
       </c>
-      <c r="G2">
-        <v>45672</v>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B3" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C3" t="str">
         <v>Invite to JRM</v>
@@ -461,18 +464,18 @@
         <v>FLCM</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G3">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B4" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -481,18 +484,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B5" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,15 +507,15 @@
         <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B6" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -521,18 +524,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B7" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -541,18 +544,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G7">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B8" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,15 +567,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,15 +587,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -601,18 +604,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -621,18 +624,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -641,21 +644,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,18 +664,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,15 +690,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -707,15 +710,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,15 +730,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -744,21 +747,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -769,16 +769,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -789,19 +792,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -816,58 +816,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -882,15 +882,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -924,16 +924,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -942,138 +945,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1085,15 +1088,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,15 +1108,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1122,95 +1125,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1406,15 +1412,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1428,10 +1434,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1542,15 +1548,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1564,27 +1570,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1596,9 +1602,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 12345
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +429,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1234</v>
+        <v>12345</v>
       </c>
       <c r="B2" t="str">
-        <v>qwer2</v>
+        <v>qew</v>
       </c>
       <c r="C2" t="str">
-        <v>qwer2</v>
+        <v>wq</v>
       </c>
       <c r="D2" t="str">
-        <v>flcm</v>
+        <v>re23</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
@@ -452,30 +452,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>1234</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>qwer2</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>qwer2</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>flcm</v>
       </c>
       <c r="E3" t="str">
         <v>jrm</v>
       </c>
-      <c r="G3">
-        <v>45672</v>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -484,18 +487,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -527,15 +530,15 @@
         <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,18 +547,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,15 +590,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B10" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -607,15 +610,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B11" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -624,18 +627,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B12" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,18 +647,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G12">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B13" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,21 +667,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F13" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G13">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B14" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,18 +687,21 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PDF</v>
       </c>
       <c r="G14">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B15" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B16" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -730,15 +733,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B17" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -750,15 +753,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B18" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -767,21 +770,18 @@
         <v>FLCM</v>
       </c>
       <c r="E18" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B19" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -792,16 +792,19 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
+      <c r="F19" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G19">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B20" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -812,19 +815,16 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
-      <c r="F20" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G20">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B21" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -839,58 +839,58 @@
         <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E22" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E23" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F23" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G23">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B25" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -928,15 +928,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B26" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -947,16 +947,19 @@
       <c r="E26" t="str">
         <v>approved</v>
       </c>
+      <c r="F26" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G26">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B27" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -965,138 +968,138 @@
         <v>FLCM</v>
       </c>
       <c r="E27" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G27">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B28" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B29" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B30" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B31" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B32" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B33" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E33" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B34" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1108,15 +1111,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B35" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1128,15 +1131,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B36" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1145,95 +1148,98 @@
         <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B37" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G37">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B38" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B39" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B40" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D40" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E40" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B41" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1242,15 +1248,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B42" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1259,15 +1265,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B43" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1276,15 +1282,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B44" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1293,15 +1299,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B45" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1310,15 +1316,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B46" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1327,15 +1333,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B47" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1344,15 +1350,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B48" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1361,15 +1367,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B49" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1378,15 +1384,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B50" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1395,15 +1401,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B51" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1412,15 +1418,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B52" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1429,15 +1435,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B53" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1451,10 +1457,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B54" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1463,15 +1469,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B55" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1480,15 +1486,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B56" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1497,15 +1503,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B57" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1514,15 +1520,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B58" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1531,15 +1537,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B59" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1548,15 +1554,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B60" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1565,15 +1571,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B61" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1587,27 +1593,27 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B62" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E62" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G62">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B63" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
@@ -1619,9 +1625,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B64" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E64" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G64">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 12323
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,30 +429,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-17062</v>
+        <v>12323</v>
       </c>
       <c r="B2" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123123</v>
       </c>
       <c r="C2" t="str">
-        <v>Invite to JRM</v>
+        <v>123123</v>
       </c>
       <c r="D2" t="str">
-        <v>FLCM</v>
+        <v>123213</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
       </c>
-      <c r="G2">
-        <v>45672</v>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B3" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C3" t="str">
         <v>Invite to JRM</v>
@@ -461,18 +464,18 @@
         <v>FLCM</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G3">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B4" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -481,18 +484,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B5" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,15 +507,15 @@
         <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B6" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -521,18 +524,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B7" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -541,18 +544,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G7">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B8" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,15 +567,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,15 +587,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -601,18 +604,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -621,18 +624,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -641,21 +644,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,18 +664,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,15 +690,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -707,15 +710,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,15 +730,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -744,21 +747,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -769,16 +769,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -789,19 +792,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -816,58 +816,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -882,15 +882,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -924,16 +924,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -942,138 +945,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1085,15 +1088,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,15 +1108,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1122,95 +1125,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1406,15 +1412,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1428,10 +1434,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1542,15 +1548,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1564,27 +1570,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1596,9 +1602,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 23434
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +429,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>12323</v>
+        <v>23434</v>
       </c>
       <c r="B2" t="str">
-        <v>123123</v>
+        <v>4324</v>
       </c>
       <c r="C2" t="str">
-        <v>123123</v>
+        <v>324</v>
       </c>
       <c r="D2" t="str">
-        <v>123213</v>
+        <v>435</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
@@ -452,30 +452,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>12323</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123123</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>123123</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>123213</v>
       </c>
       <c r="E3" t="str">
         <v>jrm</v>
       </c>
-      <c r="G3">
-        <v>45672</v>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -484,18 +487,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -527,15 +530,15 @@
         <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,18 +547,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,15 +590,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B10" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -607,15 +610,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B11" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -624,18 +627,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B12" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,18 +647,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G12">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B13" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,21 +667,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F13" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G13">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B14" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,18 +687,21 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PDF</v>
       </c>
       <c r="G14">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B15" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B16" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -730,15 +733,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B17" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -750,15 +753,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B18" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -767,21 +770,18 @@
         <v>FLCM</v>
       </c>
       <c r="E18" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B19" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -792,16 +792,19 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
+      <c r="F19" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G19">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B20" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -812,19 +815,16 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
-      <c r="F20" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G20">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B21" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -839,58 +839,58 @@
         <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E22" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E23" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F23" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G23">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B25" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -928,15 +928,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B26" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -947,16 +947,19 @@
       <c r="E26" t="str">
         <v>approved</v>
       </c>
+      <c r="F26" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G26">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B27" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -965,138 +968,138 @@
         <v>FLCM</v>
       </c>
       <c r="E27" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G27">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B28" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B29" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B30" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B31" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B32" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B33" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E33" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B34" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1108,15 +1111,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B35" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1128,15 +1131,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B36" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1145,95 +1148,98 @@
         <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B37" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G37">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B38" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B39" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B40" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D40" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E40" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B41" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1242,15 +1248,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B42" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1259,15 +1265,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B43" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1276,15 +1282,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B44" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1293,15 +1299,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B45" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1310,15 +1316,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B46" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1327,15 +1333,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B47" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1344,15 +1350,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B48" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1361,15 +1367,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B49" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1378,15 +1384,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B50" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1395,15 +1401,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B51" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1412,15 +1418,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B52" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1429,15 +1435,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B53" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1451,10 +1457,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B54" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1463,15 +1469,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B55" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1480,15 +1486,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B56" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1497,15 +1503,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B57" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1514,15 +1520,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B58" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1531,15 +1537,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B59" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1548,15 +1554,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B60" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1565,15 +1571,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B61" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1587,27 +1593,27 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B62" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E62" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G62">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B63" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
@@ -1619,9 +1625,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B64" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E64" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G64">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 123445
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>123445</v>
+      </c>
+      <c r="B2" t="str">
         <v>1234</v>
-      </c>
-      <c r="B2" t="str">
-        <v>1234123</v>
       </c>
       <c r="C2" t="str">
         <v>1234</v>
@@ -452,30 +452,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16949</v>
+        <v>1234</v>
       </c>
       <c r="B3" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>1234123</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>1234</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>1234</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G3">
-        <v>45531</v>
+        <v>jrm</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B4" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -484,18 +487,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B5" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -507,15 +510,15 @@
         <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B6" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -524,18 +527,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B7" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,18 +547,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G7">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B8" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -567,15 +570,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,15 +590,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -604,18 +607,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -624,18 +627,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,21 +647,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,18 +667,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -690,15 +693,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -730,15 +733,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -747,21 +750,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -772,16 +772,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -792,19 +795,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -819,58 +819,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -885,15 +885,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -908,15 +908,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -927,16 +927,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -945,138 +948,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1088,15 +1091,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1108,15 +1111,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1125,95 +1128,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1222,15 +1228,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1239,15 +1245,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1256,15 +1262,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1273,15 +1279,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1290,15 +1296,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1307,15 +1313,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1324,15 +1330,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1341,15 +1347,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1358,15 +1364,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1375,15 +1381,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1392,15 +1398,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1409,15 +1415,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1431,10 +1437,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1443,15 +1449,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1460,15 +1466,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1477,15 +1483,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1494,15 +1500,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1511,15 +1517,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1528,15 +1534,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1545,15 +1551,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1567,27 +1573,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1599,9 +1605,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 54354
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +429,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>123445</v>
+        <v>54354</v>
       </c>
       <c r="B2" t="str">
-        <v>1234</v>
+        <v>6546</v>
       </c>
       <c r="C2" t="str">
-        <v>1234</v>
+        <v>345</v>
       </c>
       <c r="D2" t="str">
-        <v>1234</v>
+        <v>6546</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
@@ -452,10 +452,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>123445</v>
+      </c>
+      <c r="B3" t="str">
         <v>1234</v>
-      </c>
-      <c r="B3" t="str">
-        <v>1234123</v>
       </c>
       <c r="C3" t="str">
         <v>1234</v>
@@ -475,30 +475,33 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>1234</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>1234123</v>
       </c>
       <c r="C4" t="str">
-        <v>Invite to JRM</v>
+        <v>1234</v>
       </c>
       <c r="D4" t="str">
-        <v>FLCM</v>
+        <v>1234</v>
       </c>
       <c r="E4" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G4">
-        <v>45531</v>
+        <v>jrm</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -507,18 +510,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -530,15 +533,15 @@
         <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -547,18 +550,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -567,18 +570,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -590,15 +593,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B10" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -610,15 +613,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B11" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -627,18 +630,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B12" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -647,18 +650,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G12">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B13" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,21 +670,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F13" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G13">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B14" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -690,18 +690,21 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PDF</v>
       </c>
       <c r="G14">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B15" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -713,15 +716,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B16" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -733,15 +736,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B17" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -753,15 +756,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B18" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -770,21 +773,18 @@
         <v>FLCM</v>
       </c>
       <c r="E18" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B19" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -795,16 +795,19 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
+      <c r="F19" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G19">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B20" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -815,19 +818,16 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
-      <c r="F20" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G20">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B21" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -842,58 +842,58 @@
         <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E22" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E23" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F23" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G23">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -908,15 +908,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B25" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -931,15 +931,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B26" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -950,16 +950,19 @@
       <c r="E26" t="str">
         <v>approved</v>
       </c>
+      <c r="F26" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G26">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B27" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -968,138 +971,138 @@
         <v>FLCM</v>
       </c>
       <c r="E27" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G27">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B28" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B29" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B30" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B31" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B32" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B33" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E33" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B34" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1111,15 +1114,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B35" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1131,15 +1134,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B36" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1148,95 +1151,98 @@
         <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B37" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G37">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B38" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B39" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B40" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D40" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E40" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B41" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1245,15 +1251,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B42" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1262,15 +1268,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B43" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1279,15 +1285,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B44" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1296,15 +1302,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B45" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1313,15 +1319,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B46" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1330,15 +1336,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B47" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1347,15 +1353,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B48" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1364,15 +1370,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B49" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1381,15 +1387,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B50" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1398,15 +1404,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B51" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1415,15 +1421,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B52" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1432,15 +1438,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B53" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1454,10 +1460,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B54" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1466,15 +1472,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B55" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1483,15 +1489,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B56" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1500,15 +1506,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B57" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1517,15 +1523,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B58" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1534,15 +1540,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B59" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1551,15 +1557,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B60" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1568,15 +1574,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B61" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1590,27 +1596,27 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B62" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E62" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G62">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B63" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
@@ -1622,9 +1628,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B64" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E64" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G64">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update metrics for intake ENT-18364
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -2160,74 +2160,20 @@
       <c r="A8" t="str">
         <v>ENT-18364</v>
       </c>
-      <c r="B8">
-        <v>1384999</v>
-      </c>
-      <c r="C8">
-        <v>50000</v>
-      </c>
-      <c r="D8">
-        <v>1113047</v>
-      </c>
-      <c r="E8">
-        <v>992739</v>
-      </c>
-      <c r="F8">
-        <v>248185</v>
-      </c>
-      <c r="G8">
-        <v>375</v>
-      </c>
-      <c r="H8">
-        <v>372900</v>
-      </c>
-      <c r="I8">
-        <v>22.3</v>
-      </c>
-      <c r="J8">
-        <v>26</v>
-      </c>
-      <c r="K8">
-        <v>656</v>
-      </c>
-      <c r="L8">
-        <v>633844</v>
-      </c>
-      <c r="M8">
-        <v>39.1</v>
-      </c>
-      <c r="N8">
-        <v>44.2</v>
-      </c>
-      <c r="O8">
-        <v>488</v>
-      </c>
-      <c r="P8">
-        <v>234180</v>
-      </c>
-      <c r="Q8">
-        <v>29.1</v>
-      </c>
-      <c r="R8">
-        <v>16.3</v>
-      </c>
-      <c r="T8">
-        <v>50000</v>
-      </c>
-      <c r="V8">
-        <v>3</v>
-      </c>
-      <c r="W8">
+      <c r="B8" t="str">
+        <v>Control of the group</v>
+      </c>
+      <c r="C8" t="str">
         <v>159</v>
       </c>
-      <c r="X8">
-        <v>144075</v>
-      </c>
-      <c r="Y8">
-        <v>9.5</v>
-      </c>
-      <c r="Z8">
-        <v>10</v>
+      <c r="D8" t="str">
+        <v>$144075</v>
+      </c>
+      <c r="E8" t="str">
+        <v>9.50%</v>
+      </c>
+      <c r="F8" t="str">
+        <v>10.00%</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update metrics for intake ENT-14372
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -2080,74 +2080,80 @@
       <c r="A7" t="str">
         <v>ENT-14372</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="str">
         <v>244153</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
+      <c r="C7" t="str">
+        <v>-</v>
+      </c>
+      <c r="D7" t="str">
+        <v>-</v>
+      </c>
+      <c r="E7" t="str">
+        <v>-</v>
+      </c>
+      <c r="F7" t="str">
+        <v>-</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-</v>
+      </c>
+      <c r="H7" t="str">
+        <v>-</v>
+      </c>
+      <c r="I7" t="str">
+        <v>-</v>
+      </c>
+      <c r="J7" t="str">
+        <v>-</v>
+      </c>
+      <c r="K7" t="str">
         <v>165</v>
       </c>
-      <c r="L7">
-        <v>127692</v>
-      </c>
-      <c r="M7">
-        <v>46.8</v>
-      </c>
-      <c r="N7">
-        <v>52.3</v>
-      </c>
-      <c r="O7">
+      <c r="L7" t="str">
+        <v>$127692</v>
+      </c>
+      <c r="M7" t="str">
+        <v>46.80%</v>
+      </c>
+      <c r="N7" t="str">
+        <v>52.30%</v>
+      </c>
+      <c r="O7" t="str">
         <v>147</v>
       </c>
-      <c r="P7">
-        <v>79763</v>
-      </c>
-      <c r="Q7">
-        <v>41.7</v>
-      </c>
-      <c r="R7">
-        <v>32.7</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
+      <c r="P7" t="str">
+        <v>$79763</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>41.70%</v>
+      </c>
+      <c r="R7" t="str">
+        <v>32.70%</v>
+      </c>
+      <c r="S7" t="str">
+        <v>-</v>
+      </c>
+      <c r="T7" t="str">
+        <v>-</v>
+      </c>
+      <c r="U7" t="str">
+        <v>-</v>
+      </c>
+      <c r="V7" t="str">
+        <v>-</v>
+      </c>
+      <c r="W7" t="str">
         <v>41</v>
       </c>
-      <c r="X7">
-        <v>36698</v>
-      </c>
-      <c r="Y7">
-        <v>11.5</v>
-      </c>
-      <c r="Z7">
-        <v>15</v>
+      <c r="X7" t="str">
+        <v>$36698</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>11.50%</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>15.00%</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Update metrics for intake ENT-17213
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1778,77 +1778,80 @@
       <c r="A3" t="str">
         <v>ENT-17213</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="str">
         <v>703188</v>
       </c>
-      <c r="C3">
-        <v>67500</v>
-      </c>
-      <c r="E3">
-        <v>425495</v>
-      </c>
-      <c r="F3">
+      <c r="C3" t="str">
+        <v>1324</v>
+      </c>
+      <c r="D3" t="str">
+        <v>-</v>
+      </c>
+      <c r="E3" t="str">
+        <v>4324</v>
+      </c>
+      <c r="F3" t="str">
         <v>106374</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="str">
         <v>159</v>
       </c>
-      <c r="H3">
-        <v>157861</v>
-      </c>
-      <c r="I3">
-        <v>14</v>
-      </c>
-      <c r="J3">
-        <v>20.5</v>
-      </c>
-      <c r="K3">
+      <c r="H3" t="str">
+        <v>$157861</v>
+      </c>
+      <c r="I3" t="str">
+        <v>120%</v>
+      </c>
+      <c r="J3" t="str">
+        <v>20.50%</v>
+      </c>
+      <c r="K3" t="str">
         <v>598</v>
       </c>
-      <c r="L3">
-        <v>308479</v>
-      </c>
-      <c r="M3">
-        <v>52.8</v>
-      </c>
-      <c r="N3">
-        <v>40</v>
-      </c>
-      <c r="O3">
+      <c r="L3" t="str">
+        <v>$308479</v>
+      </c>
+      <c r="M3" t="str">
+        <v>52.80%</v>
+      </c>
+      <c r="N3" t="str">
+        <v>40.00%</v>
+      </c>
+      <c r="O3" t="str">
         <v>303</v>
       </c>
-      <c r="P3">
-        <v>158200</v>
-      </c>
-      <c r="Q3">
-        <v>26.7</v>
-      </c>
-      <c r="R3">
-        <v>20.5</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <v>50000</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
+      <c r="P3" t="str">
+        <v>$158200</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>26.70%</v>
+      </c>
+      <c r="R3" t="str">
+        <v>20.50%</v>
+      </c>
+      <c r="S3" t="str">
+        <v>-</v>
+      </c>
+      <c r="T3" t="str">
+        <v>$50000</v>
+      </c>
+      <c r="U3" t="str">
+        <v>-</v>
+      </c>
+      <c r="V3" t="str">
+        <v>-</v>
+      </c>
+      <c r="W3" t="str">
         <v>73</v>
       </c>
-      <c r="X3">
-        <v>78648</v>
-      </c>
-      <c r="Y3">
-        <v>6.4</v>
-      </c>
-      <c r="Z3">
-        <v>10.2</v>
+      <c r="X3" t="str">
+        <v>$78648</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>6.40%</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>10.20%</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Update Metrics row for ENT-17213
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1791,7 +1791,7 @@
         <v>106374</v>
       </c>
       <c r="G3" t="str">
-        <v>160</v>
+        <v>700</v>
       </c>
       <c r="H3" t="str">
         <v>157861</v>
@@ -1800,7 +1800,7 @@
         <v>14.00</v>
       </c>
       <c r="J3" t="str">
-        <v>200</v>
+        <v>200.00</v>
       </c>
       <c r="K3">
         <v>598</v>

</xml_diff>

<commit_message>
Update Metrics row for ENT-17054
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1713,17 +1713,17 @@
       <c r="F2">
         <v>59466</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="str">
         <v>90</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="str">
         <v>83903</v>
       </c>
-      <c r="I2">
-        <v>38.7</v>
-      </c>
-      <c r="J2">
-        <v>46.4</v>
+      <c r="I2" t="str">
+        <v>38.70</v>
+      </c>
+      <c r="J2" t="str">
+        <v>46.40</v>
       </c>
       <c r="K2">
         <v>68</v>
@@ -1749,17 +1749,17 @@
       <c r="R2">
         <v>20.6</v>
       </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
+      <c r="S2" t="str">
+        <v>-</v>
+      </c>
+      <c r="T2" t="str">
         <v>2500</v>
       </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>1</v>
+      <c r="U2" t="str">
+        <v>-</v>
+      </c>
+      <c r="V2" t="str">
+        <v>100.34</v>
       </c>
       <c r="W2">
         <v>0</v>

</xml_diff>

<commit_message>
Add new intake 17062
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,30 +429,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-17062</v>
+        <v>17062</v>
       </c>
       <c r="B2" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123</v>
       </c>
       <c r="C2" t="str">
-        <v>Invite to JRM</v>
+        <v>123</v>
       </c>
       <c r="D2" t="str">
-        <v>FLCM</v>
+        <v>123</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
       </c>
-      <c r="G2">
-        <v>45672</v>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B3" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C3" t="str">
         <v>Invite to JRM</v>
@@ -461,18 +464,18 @@
         <v>FLCM</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G3">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B4" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -481,18 +484,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B5" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,15 +507,15 @@
         <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B6" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -521,18 +524,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B7" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -541,18 +544,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G7">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B8" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,15 +567,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,15 +587,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -601,18 +604,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -621,18 +624,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -641,21 +644,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,18 +664,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,15 +690,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -707,15 +710,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,15 +730,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -744,21 +747,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -769,16 +769,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -789,19 +792,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -816,58 +816,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -882,15 +882,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -924,16 +924,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -942,138 +945,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1085,15 +1088,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,15 +1108,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1122,95 +1125,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1406,15 +1412,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1428,10 +1434,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1542,15 +1548,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1564,27 +1570,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1596,19 +1602,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F12" r:id="rId1"/>
-    <hyperlink ref="F17" r:id="rId2"/>
-    <hyperlink ref="F19" r:id="rId3"/>
-    <hyperlink ref="F20" r:id="rId4"/>
-    <hyperlink ref="F22" r:id="rId5"/>
-    <hyperlink ref="F23" r:id="rId6"/>
-    <hyperlink ref="F24" r:id="rId7"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake ENT-168812
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>17062</v>
+        <v>ENT-168812</v>
       </c>
       <c r="B2" t="str">
-        <v>123</v>
+        <v>terw</v>
       </c>
       <c r="C2" t="str">
         <v>123</v>
@@ -452,30 +452,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>17062</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>123</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>123</v>
       </c>
       <c r="E3" t="str">
         <v>jrm</v>
       </c>
-      <c r="G3">
-        <v>45672</v>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -484,18 +487,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -527,15 +530,15 @@
         <v>jrm</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,18 +547,18 @@
         <v>FLCM</v>
       </c>
       <c r="E7" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,15 +590,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B10" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -607,15 +610,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B11" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -624,18 +627,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B12" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,18 +647,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G12">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B13" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,21 +667,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F13" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G13">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B14" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,18 +687,21 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PDF</v>
       </c>
       <c r="G14">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B15" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B16" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -730,15 +733,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B17" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -750,15 +753,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B18" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -767,21 +770,18 @@
         <v>FLCM</v>
       </c>
       <c r="E18" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B19" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -792,16 +792,19 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
+      <c r="F19" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G19">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B20" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -812,19 +815,16 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
-      <c r="F20" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G20">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B21" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -839,58 +839,58 @@
         <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E22" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E23" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F23" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G23">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B25" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -928,15 +928,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B26" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -947,16 +947,19 @@
       <c r="E26" t="str">
         <v>approved</v>
       </c>
+      <c r="F26" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G26">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B27" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -965,138 +968,138 @@
         <v>FLCM</v>
       </c>
       <c r="E27" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G27">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B28" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B29" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B30" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B31" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B32" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B33" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E33" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B34" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1108,15 +1111,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B35" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1128,15 +1131,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B36" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1145,95 +1148,98 @@
         <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B37" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G37">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B38" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B39" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B40" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D40" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E40" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B41" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1242,15 +1248,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B42" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1259,15 +1265,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B43" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1276,15 +1282,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B44" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1293,15 +1299,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B45" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1310,15 +1316,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B46" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1327,15 +1333,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B47" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1344,15 +1350,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B48" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1361,15 +1367,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B49" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1378,15 +1384,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B50" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1395,15 +1401,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B51" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1412,15 +1418,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B52" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1429,15 +1435,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B53" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1451,10 +1457,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B54" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1463,15 +1469,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B55" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1480,15 +1486,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B56" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1497,15 +1503,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B57" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1514,15 +1520,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B58" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1531,15 +1537,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B59" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1548,15 +1554,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B60" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1565,15 +1571,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B61" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1587,27 +1593,27 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B62" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E62" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G62">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B63" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
@@ -1619,9 +1625,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B64" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E64" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G64">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake ENT-168843
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +429,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-168812</v>
+        <v>ENT-168843</v>
       </c>
       <c r="B2" t="str">
-        <v>terw</v>
+        <v>qwe</v>
       </c>
       <c r="C2" t="str">
-        <v>123</v>
+        <v>qwe</v>
       </c>
       <c r="D2" t="str">
-        <v>123</v>
+        <v>qwe</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
@@ -452,10 +452,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>17062</v>
+        <v>ENT-168812</v>
       </c>
       <c r="B3" t="str">
-        <v>123</v>
+        <v>terw</v>
       </c>
       <c r="C3" t="str">
         <v>123</v>
@@ -475,30 +475,33 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-17062</v>
+        <v>17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123</v>
       </c>
       <c r="C4" t="str">
-        <v>Invite to JRM</v>
+        <v>123</v>
       </c>
       <c r="D4" t="str">
-        <v>FLCM</v>
+        <v>123</v>
       </c>
       <c r="E4" t="str">
         <v>jrm</v>
       </c>
-      <c r="G4">
-        <v>45672</v>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B5" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -507,18 +510,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B6" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -527,18 +530,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G6">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B7" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -550,15 +553,15 @@
         <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B8" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -567,18 +570,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B9" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,18 +590,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G9">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B10" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -610,15 +613,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B11" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -630,15 +633,15 @@
         <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B12" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -647,18 +650,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B13" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,18 +670,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G13">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B14" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,21 +690,18 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F14" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G14">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B15" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,18 +710,21 @@
         <v>FLCM</v>
       </c>
       <c r="E15" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PDF</v>
       </c>
       <c r="G15">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B16" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -733,15 +736,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B17" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -753,15 +756,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B18" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -773,15 +776,15 @@
         <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B19" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -790,21 +793,18 @@
         <v>FLCM</v>
       </c>
       <c r="E19" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G19">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B20" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -815,16 +815,19 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
+      <c r="F20" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G20">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B21" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -835,19 +838,16 @@
       <c r="E21" t="str">
         <v>approved</v>
       </c>
-      <c r="F21" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G21">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B22" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
@@ -862,58 +862,58 @@
         <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E23" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B24" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D24" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E24" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F24" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G24">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -928,15 +928,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B26" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -951,15 +951,15 @@
         <v>PDF</v>
       </c>
       <c r="G26">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B27" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -970,16 +970,19 @@
       <c r="E27" t="str">
         <v>approved</v>
       </c>
+      <c r="F27" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G27">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B28" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
@@ -988,138 +991,138 @@
         <v>FLCM</v>
       </c>
       <c r="E28" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G28">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B29" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B30" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B31" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B32" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B33" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E33" t="str">
         <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B34" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D34" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E34" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G34">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B35" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1131,15 +1134,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B36" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1151,15 +1154,15 @@
         <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B37" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
@@ -1168,95 +1171,98 @@
         <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G37">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B38" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G38">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B39" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B40" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D40" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E40" t="str">
         <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B41" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D41" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E41" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G41">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B42" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1265,15 +1271,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B43" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1282,15 +1288,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B44" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1299,15 +1305,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B45" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1316,15 +1322,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B46" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1333,15 +1339,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B47" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1350,15 +1356,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B48" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1367,15 +1373,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B49" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1384,15 +1390,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B50" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1401,15 +1407,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B51" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1418,15 +1424,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B52" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1435,15 +1441,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B53" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1452,15 +1458,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B54" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1474,10 +1480,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B55" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1486,15 +1492,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B56" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1503,15 +1509,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B57" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1520,15 +1526,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B58" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1537,15 +1543,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B59" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1554,15 +1560,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B60" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1571,15 +1577,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B61" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1588,15 +1594,15 @@
         <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B62" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1610,27 +1616,27 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B63" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E63" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G63">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B64" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C64" t="str">
         <v>Invite to JRM</v>
@@ -1642,9 +1648,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B65" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E65" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G65">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G65"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 234234
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +429,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-168812</v>
+        <v>234234</v>
       </c>
       <c r="B2" t="str">
-        <v>terw</v>
+        <v>5345</v>
       </c>
       <c r="C2" t="str">
-        <v>123</v>
+        <v>345</v>
       </c>
       <c r="D2" t="str">
-        <v>123</v>
+        <v>345345</v>
       </c>
       <c r="E2" t="str">
         <v>jrm</v>
@@ -447,15 +447,15 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2025-03-15</v>
+        <v>2025-03-16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>17062</v>
+        <v>ENT-168812</v>
       </c>
       <c r="B3" t="str">
-        <v>123</v>
+        <v>terw</v>
       </c>
       <c r="C3" t="str">
         <v>123</v>
@@ -475,30 +475,33 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-17062</v>
+        <v>17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>123</v>
       </c>
       <c r="C4" t="str">
-        <v>Invite to JRM</v>
+        <v>123</v>
       </c>
       <c r="D4" t="str">
-        <v>FLCM</v>
+        <v>123</v>
       </c>
       <c r="E4" t="str">
         <v>jrm</v>
       </c>
-      <c r="G4">
-        <v>45672</v>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2025-03-15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B5" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -507,18 +510,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G5">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B6" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -527,18 +530,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G6">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B7" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -550,15 +553,15 @@
         <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B8" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -567,18 +570,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B9" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -587,18 +590,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G9">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B10" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -610,15 +613,15 @@
         <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B11" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -630,15 +633,15 @@
         <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B12" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -647,18 +650,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B13" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,18 +670,18 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G13">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B14" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,21 +690,18 @@
         <v>FLCM</v>
       </c>
       <c r="E14" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F14" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G14">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B15" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,18 +710,21 @@
         <v>FLCM</v>
       </c>
       <c r="E15" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PDF</v>
       </c>
       <c r="G15">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B16" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -733,15 +736,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B17" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -753,15 +756,15 @@
         <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B18" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -773,15 +776,15 @@
         <v>estimates</v>
       </c>
       <c r="G18">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B19" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -790,21 +793,18 @@
         <v>FLCM</v>
       </c>
       <c r="E19" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G19">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B20" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -815,16 +815,19 @@
       <c r="E20" t="str">
         <v>approved</v>
       </c>
+      <c r="F20" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G20">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B21" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
@@ -835,19 +838,16 @@
       <c r="E21" t="str">
         <v>approved</v>
       </c>
-      <c r="F21" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G21">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B22" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
@@ -862,58 +862,58 @@
         <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B23" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D23" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E23" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B24" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D24" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E24" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F24" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G24">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -928,15 +928,15 @@
         <v>PDF</v>
       </c>
       <c r="G25">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B26" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -951,15 +951,15 @@
         <v>PDF</v>
       </c>
       <c r="G26">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B27" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
@@ -970,16 +970,19 @@
       <c r="E27" t="str">
         <v>approved</v>
       </c>
+      <c r="F27" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G27">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B28" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
@@ -988,138 +991,138 @@
         <v>FLCM</v>
       </c>
       <c r="E28" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G28">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B29" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B30" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B31" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B32" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E32" t="str">
         <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B33" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D33" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E33" t="str">
         <v>estimates</v>
       </c>
       <c r="G33">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B34" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D34" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E34" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G34">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B35" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1131,15 +1134,15 @@
         <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B36" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
@@ -1151,15 +1154,15 @@
         <v>ofs</v>
       </c>
       <c r="G36">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B37" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
@@ -1168,95 +1171,98 @@
         <v>FLCM</v>
       </c>
       <c r="E37" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G37">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B38" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G38">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B39" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D39" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E39" t="str">
         <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B40" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D40" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E40" t="str">
         <v>estimates</v>
       </c>
       <c r="G40">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B41" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D41" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E41" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G41">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B42" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1265,15 +1271,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B43" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1282,15 +1288,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B44" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1299,15 +1305,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B45" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1316,15 +1322,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B46" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1333,15 +1339,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B47" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1350,15 +1356,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B48" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1367,15 +1373,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B49" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1384,15 +1390,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B50" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1401,15 +1407,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B51" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1418,15 +1424,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B52" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1435,15 +1441,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B53" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1452,15 +1458,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B54" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1474,10 +1480,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B55" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1486,15 +1492,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B56" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1503,15 +1509,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B57" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1520,15 +1526,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B58" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1537,15 +1543,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B59" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1554,15 +1560,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B60" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1571,15 +1577,15 @@
         <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B61" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1588,15 +1594,15 @@
         <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B62" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1610,27 +1616,27 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B63" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C63" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E63" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G63">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B64" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C64" t="str">
         <v>Invite to JRM</v>
@@ -1642,9 +1648,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B65" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E65" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G65">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G65"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update Metrics row for ENT-17705
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1999,17 +1999,20 @@
       <c r="A6" t="str">
         <v>ENT-17705</v>
       </c>
-      <c r="B6">
-        <v>46433</v>
-      </c>
-      <c r="C6">
-        <v>5000</v>
-      </c>
-      <c r="E6">
-        <v>30962</v>
-      </c>
-      <c r="F6">
-        <v>15481</v>
+      <c r="B6" t="str">
+        <v>46433.00</v>
+      </c>
+      <c r="C6" t="str">
+        <v>5000.00</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>30962.00</v>
+      </c>
+      <c r="F6" t="str">
+        <v>4234234</v>
       </c>
       <c r="G6">
         <v>23</v>

</xml_diff>

<commit_message>
Add new intake 435
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,30 +429,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-17062</v>
+        <v>435</v>
       </c>
       <c r="B2" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>345</v>
       </c>
       <c r="C2" t="str">
-        <v>Invite to JRM</v>
+        <v>345</v>
       </c>
       <c r="D2" t="str">
-        <v>FLCM</v>
+        <v>345345</v>
       </c>
       <c r="E2" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G2">
-        <v>45672</v>
+        <v>jrm</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-01</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B3" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C3" t="str">
         <v>Invite to JRM</v>
@@ -464,15 +467,15 @@
         <v>estimates</v>
       </c>
       <c r="G3">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B4" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -481,18 +484,18 @@
         <v>FLCM</v>
       </c>
       <c r="E4" t="str">
-        <v>approved</v>
+        <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B5" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -501,18 +504,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>ofs</v>
+        <v>approved</v>
       </c>
       <c r="G5">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B6" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -521,18 +524,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G6">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B7" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,15 +547,15 @@
         <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B8" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,15 +567,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,15 +587,15 @@
         <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -601,18 +604,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -621,18 +624,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -641,21 +644,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -664,18 +664,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,15 +690,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -707,15 +710,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,15 +730,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -744,21 +747,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -769,16 +769,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -789,19 +792,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -816,58 +816,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -882,15 +882,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -905,15 +905,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -924,16 +924,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -942,138 +945,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1085,15 +1088,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,15 +1108,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1122,95 +1125,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1406,15 +1412,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1428,10 +1434,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1542,15 +1548,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1564,27 +1570,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1596,9 +1602,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 16031
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,53 +429,56 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>435</v>
+        <v>16031</v>
       </c>
       <c r="B2" t="str">
-        <v>345</v>
+        <v>qweqwe</v>
       </c>
       <c r="C2" t="str">
-        <v>345</v>
+        <v>qweqwe</v>
       </c>
       <c r="D2" t="str">
-        <v>345345</v>
+        <v>qweqwe</v>
       </c>
       <c r="E2" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2025-03-01</v>
+        <v>2025-03-04</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>435</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>345</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>345</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>345345</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G3">
-        <v>45672</v>
+        <v>approved</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-01</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -487,15 +490,15 @@
         <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>approved</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -524,18 +527,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>ofs</v>
+        <v>approved</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -547,15 +550,15 @@
         <v>ofs</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>estimates</v>
+        <v>ofs</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,18 +587,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -604,18 +607,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -624,18 +627,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G11">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B12" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,21 +647,18 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F12" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G12">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B13" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,18 +667,21 @@
         <v>FLCM</v>
       </c>
       <c r="E13" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PDF</v>
       </c>
       <c r="G13">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B14" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -690,15 +693,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B15" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B16" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -730,15 +733,15 @@
         <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B17" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -747,21 +750,18 @@
         <v>FLCM</v>
       </c>
       <c r="E17" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F17" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G17">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B18" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -772,16 +772,19 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
+      <c r="F18" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G18">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B19" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -792,19 +795,16 @@
       <c r="E19" t="str">
         <v>approved</v>
       </c>
-      <c r="F19" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G19">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B20" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
@@ -819,58 +819,58 @@
         <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E21" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PDF</v>
       </c>
       <c r="G21">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B22" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D22" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E22" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G22">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B23" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -885,15 +885,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B24" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -908,15 +908,15 @@
         <v>PDF</v>
       </c>
       <c r="G24">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B25" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -927,16 +927,19 @@
       <c r="E25" t="str">
         <v>approved</v>
       </c>
+      <c r="F25" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G25">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B26" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
@@ -945,138 +948,138 @@
         <v>FLCM</v>
       </c>
       <c r="E26" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G26">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B27" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B28" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B29" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B30" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B31" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E31" t="str">
         <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B32" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D32" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E32" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G32">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B33" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1088,15 +1091,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B34" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1108,15 +1111,15 @@
         <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B35" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
@@ -1125,95 +1128,98 @@
         <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G35">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B36" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E36" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G36">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B37" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B38" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D38" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E38" t="str">
         <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B39" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D39" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E39" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G39">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B40" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1222,15 +1228,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B41" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1239,15 +1245,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B42" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1256,15 +1262,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B43" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1273,15 +1279,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B44" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1290,15 +1296,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B45" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1307,15 +1313,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B46" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1324,15 +1330,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B47" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1341,15 +1347,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B48" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1358,15 +1364,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B49" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1375,15 +1381,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B50" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1392,15 +1398,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B51" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1409,15 +1415,15 @@
         <v>ofs</v>
       </c>
       <c r="G51">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B52" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1431,10 +1437,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B53" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1443,15 +1449,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B54" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1460,15 +1466,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B55" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1477,15 +1483,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B56" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1494,15 +1500,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B57" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1511,15 +1517,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B58" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1528,15 +1534,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B59" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1545,15 +1551,15 @@
         <v>ofs</v>
       </c>
       <c r="G59">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B60" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
@@ -1567,27 +1573,27 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B61" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E61" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G61">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B62" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C62" t="str">
         <v>Invite to JRM</v>
@@ -1599,9 +1605,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B63" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E63" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G63">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 2123
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,53 +429,56 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>16031</v>
+        <v>2123</v>
       </c>
       <c r="B2" t="str">
-        <v>qweqwe</v>
+        <v>234234</v>
       </c>
       <c r="C2" t="str">
-        <v>qweqwe</v>
+        <v>234234</v>
       </c>
       <c r="D2" t="str">
-        <v>qweqwe</v>
+        <v>234234</v>
       </c>
       <c r="E2" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2025-03-04</v>
+        <v>2025-02-26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>16031</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>qweqwe</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>qweqwe</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>qweqwe</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G3">
-        <v>45672</v>
+        <v>approved</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-04</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -487,15 +490,15 @@
         <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>approved</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -524,18 +527,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>ofs</v>
+        <v>approved</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -547,15 +550,15 @@
         <v>ofs</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>estimates</v>
+        <v>ofs</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,18 +587,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>jrm</v>
+        <v>estimates</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -604,18 +607,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -626,19 +629,16 @@
       <c r="E11" t="str">
         <v>approved</v>
       </c>
-      <c r="F11" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G11">
-        <v>45686</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B12" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -647,18 +647,21 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PDF</v>
       </c>
       <c r="G12">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B13" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -670,15 +673,15 @@
         <v>estimates</v>
       </c>
       <c r="G13">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B14" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -690,15 +693,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B15" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B16" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,21 +730,18 @@
         <v>FLCM</v>
       </c>
       <c r="E16" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F16" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B17" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -752,16 +752,19 @@
       <c r="E17" t="str">
         <v>approved</v>
       </c>
+      <c r="F17" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G17">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B18" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -772,19 +775,16 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G18">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B19" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -799,58 +799,58 @@
         <v>PDF</v>
       </c>
       <c r="G19">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B20" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D20" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E20" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E21" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F21" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G21">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B22" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
@@ -865,15 +865,15 @@
         <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B23" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -888,15 +888,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -907,16 +907,19 @@
       <c r="E24" t="str">
         <v>approved</v>
       </c>
+      <c r="F24" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G24">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B25" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -925,138 +928,138 @@
         <v>FLCM</v>
       </c>
       <c r="E25" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G25">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B26" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D26" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E26" t="str">
         <v>estimates</v>
       </c>
       <c r="G26">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B27" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B28" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B29" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B30" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B31" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E31" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B32" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
@@ -1068,15 +1071,15 @@
         <v>ofs</v>
       </c>
       <c r="G32">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B33" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1088,15 +1091,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B34" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,95 +1108,98 @@
         <v>FLCM</v>
       </c>
       <c r="E34" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B35" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D35" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G35">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B36" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E36" t="str">
         <v>estimates</v>
       </c>
       <c r="G36">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B37" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B38" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D38" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E38" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B39" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
@@ -1202,15 +1208,15 @@
         <v>ofs</v>
       </c>
       <c r="G39">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B40" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B41" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B42" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B43" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B44" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B45" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B46" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B47" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B48" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B49" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B50" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B51" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1411,10 +1417,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B52" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1423,15 +1429,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B53" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B54" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B55" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B56" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B57" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B58" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B59" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1547,27 +1553,27 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B60" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E60" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B61" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1579,9 +1585,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B62" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E62" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G62">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 18472
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,53 +429,56 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>16031</v>
+        <v>18472</v>
       </c>
       <c r="B2" t="str">
-        <v>qweqwe</v>
+        <v>12321</v>
       </c>
       <c r="C2" t="str">
-        <v>qweqwe</v>
+        <v>123123</v>
       </c>
       <c r="D2" t="str">
-        <v>qweqwe</v>
+        <v>123123</v>
       </c>
       <c r="E2" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2025-03-04</v>
+        <v>2025-03-10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-17062</v>
+        <v>16031</v>
       </c>
       <c r="B3" t="str">
-        <v>Account Open Enhancements and Outcome Orchestration</v>
+        <v>qweqwe</v>
       </c>
       <c r="C3" t="str">
-        <v>Invite to JRM</v>
+        <v>qweqwe</v>
       </c>
       <c r="D3" t="str">
-        <v>FLCM</v>
+        <v>qweqwe</v>
       </c>
       <c r="E3" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G3">
-        <v>45672</v>
+        <v>approved</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2025-03-04</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16949</v>
+        <v>ENT-17062</v>
       </c>
       <c r="B4" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>Account Open Enhancements and Outcome Orchestration</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -487,15 +490,15 @@
         <v>estimates</v>
       </c>
       <c r="G4">
-        <v>45531</v>
+        <v>45672</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B5" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,18 +507,18 @@
         <v>FLCM</v>
       </c>
       <c r="E5" t="str">
-        <v>approved</v>
+        <v>estimates</v>
       </c>
       <c r="G5">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B6" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -524,18 +527,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>ofs</v>
+        <v>approved</v>
       </c>
       <c r="G6">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B7" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -547,15 +550,15 @@
         <v>ofs</v>
       </c>
       <c r="G7">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B8" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,18 +567,18 @@
         <v>FLCM</v>
       </c>
       <c r="E8" t="str">
-        <v>estimates</v>
+        <v>ofs</v>
       </c>
       <c r="G8">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B9" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -584,18 +587,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G9">
-        <v>45613</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B10" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -604,18 +607,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>approved</v>
+        <v>ofs</v>
       </c>
       <c r="G10">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B11" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -626,19 +629,16 @@
       <c r="E11" t="str">
         <v>approved</v>
       </c>
-      <c r="F11" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G11">
-        <v>45686</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B12" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -647,18 +647,21 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PDF</v>
       </c>
       <c r="G12">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B13" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -670,15 +673,15 @@
         <v>estimates</v>
       </c>
       <c r="G13">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B14" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -690,15 +693,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B15" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -710,15 +713,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B16" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -727,21 +730,18 @@
         <v>FLCM</v>
       </c>
       <c r="E16" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F16" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B17" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -752,16 +752,19 @@
       <c r="E17" t="str">
         <v>approved</v>
       </c>
+      <c r="F17" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G17">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B18" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -772,19 +775,16 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G18">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B19" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -799,58 +799,58 @@
         <v>PDF</v>
       </c>
       <c r="G19">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B20" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D20" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E20" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E21" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F21" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G21">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B22" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
@@ -865,15 +865,15 @@
         <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B23" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -888,15 +888,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -907,16 +907,19 @@
       <c r="E24" t="str">
         <v>approved</v>
       </c>
+      <c r="F24" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G24">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B25" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -925,138 +928,138 @@
         <v>FLCM</v>
       </c>
       <c r="E25" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G25">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B26" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D26" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E26" t="str">
         <v>estimates</v>
       </c>
       <c r="G26">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B27" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B28" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B29" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B30" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B31" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E31" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B32" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
@@ -1068,15 +1071,15 @@
         <v>ofs</v>
       </c>
       <c r="G32">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B33" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1088,15 +1091,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B34" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1105,95 +1108,98 @@
         <v>FLCM</v>
       </c>
       <c r="E34" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B35" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D35" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G35">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B36" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E36" t="str">
         <v>estimates</v>
       </c>
       <c r="G36">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B37" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B38" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D38" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E38" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B39" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
@@ -1202,15 +1208,15 @@
         <v>ofs</v>
       </c>
       <c r="G39">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B40" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1219,15 +1225,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B41" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1236,15 +1242,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B42" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1253,15 +1259,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B43" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1270,15 +1276,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B44" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1287,15 +1293,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B45" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1304,15 +1310,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B46" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1321,15 +1327,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B47" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1338,15 +1344,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B48" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1355,15 +1361,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B49" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1372,15 +1378,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B50" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1389,15 +1395,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B51" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1411,10 +1417,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B52" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1423,15 +1429,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B53" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1440,15 +1446,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B54" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1457,15 +1463,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B55" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1474,15 +1480,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B56" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1491,15 +1497,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B57" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1508,15 +1514,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B58" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1525,15 +1531,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B59" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1547,27 +1553,27 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B60" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E60" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B61" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1579,9 +1585,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B62" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E62" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G62">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new intake 12344
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,30 +429,33 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ENT-16949</v>
+        <v>12344</v>
       </c>
       <c r="B2" t="str">
-        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
+        <v>324</v>
       </c>
       <c r="C2" t="str">
-        <v>Invite to JRM</v>
+        <v>234234</v>
       </c>
       <c r="D2" t="str">
-        <v>FLCM</v>
+        <v>234234</v>
       </c>
       <c r="E2" t="str">
-        <v>estimates</v>
-      </c>
-      <c r="G2">
-        <v>45531</v>
+        <v>jrm</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2025-03-10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-16949</v>
       </c>
       <c r="B3" t="str">
-        <v>Split up Personal Overdraft P&amp;L</v>
+        <v>Fusion: CSP Cards Status Frequency Update-RBSSINTK-9334</v>
       </c>
       <c r="C3" t="str">
         <v>Invite to JRM</v>
@@ -461,18 +464,18 @@
         <v>FLCM</v>
       </c>
       <c r="E3" t="str">
-        <v>approved</v>
+        <v>estimates</v>
       </c>
       <c r="G3">
-        <v>45929</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ENT-16700</v>
+        <v>ENT-16881</v>
       </c>
       <c r="B4" t="str">
-        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
+        <v>Split up Personal Overdraft P&amp;L</v>
       </c>
       <c r="C4" t="str">
         <v>Invite to JRM</v>
@@ -484,15 +487,15 @@
         <v>approved</v>
       </c>
       <c r="G4">
-        <v>45523</v>
+        <v>45929</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ENT-16621</v>
+        <v>ENT-16700</v>
       </c>
       <c r="B5" t="str">
-        <v>CIW Data Products to PROD</v>
+        <v>Simplii Debit Mastercard (Debit Card) MCC Block Removal</v>
       </c>
       <c r="C5" t="str">
         <v>Invite to JRM</v>
@@ -504,15 +507,15 @@
         <v>approved</v>
       </c>
       <c r="G5">
-        <v>45596</v>
+        <v>45523</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENT-16374</v>
+        <v>ENT-16621</v>
       </c>
       <c r="B6" t="str">
-        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
+        <v>CIW Data Products to PROD</v>
       </c>
       <c r="C6" t="str">
         <v>Invite to JRM</v>
@@ -521,18 +524,18 @@
         <v>FLCM</v>
       </c>
       <c r="E6" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G6">
-        <v>45455</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENT-16031</v>
+        <v>ENT-16374</v>
       </c>
       <c r="B7" t="str">
-        <v>Fraud - Notes generator</v>
+        <v>eBIT Migration Account Open Initiative: Citadel Estimates</v>
       </c>
       <c r="C7" t="str">
         <v>Invite to JRM</v>
@@ -544,15 +547,15 @@
         <v>jrm</v>
       </c>
       <c r="G7">
-        <v>45649</v>
+        <v>45455</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ENT-15917</v>
+        <v>ENT-16031</v>
       </c>
       <c r="B8" t="str">
-        <v>REBO Bill Payment Investigation Requests</v>
+        <v>Fraud - Notes generator</v>
       </c>
       <c r="C8" t="str">
         <v>Invite to JRM</v>
@@ -564,15 +567,15 @@
         <v>jrm</v>
       </c>
       <c r="G8">
-        <v>45613</v>
+        <v>45649</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-17286</v>
+        <v>ENT-15917</v>
       </c>
       <c r="B9" t="str">
-        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
+        <v>REBO Bill Payment Investigation Requests</v>
       </c>
       <c r="C9" t="str">
         <v>Invite to JRM</v>
@@ -581,18 +584,18 @@
         <v>FLCM</v>
       </c>
       <c r="E9" t="str">
-        <v>approved</v>
+        <v>jrm</v>
       </c>
       <c r="G9">
-        <v>45699</v>
+        <v>45613</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ENT-17202</v>
+        <v>ENT-17286</v>
       </c>
       <c r="B10" t="str">
-        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
+        <v>SAS Viya HMS High Level Estimates- FY 25 and FY 26</v>
       </c>
       <c r="C10" t="str">
         <v>Invite to JRM</v>
@@ -601,18 +604,18 @@
         <v>FLCM</v>
       </c>
       <c r="E10" t="str">
-        <v>jrm</v>
+        <v>approved</v>
       </c>
       <c r="G10">
-        <v>45690</v>
+        <v>45699</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ENT-18364</v>
+        <v>ENT-17202</v>
       </c>
       <c r="B11" t="str">
-        <v>Expansion of US FCM for US Payments</v>
+        <v>EDH to EDGE Consumption Migration for Fraud teams</v>
       </c>
       <c r="C11" t="str">
         <v>Invite to JRM</v>
@@ -621,21 +624,18 @@
         <v>FLCM</v>
       </c>
       <c r="E11" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F11" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G11">
-        <v>45686</v>
+        <v>45690</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ENT-17639</v>
+        <v>ENT-18364</v>
       </c>
       <c r="B12" t="str">
-        <v>Send DAC ID to FIQM</v>
+        <v>Expansion of US FCM for US Payments</v>
       </c>
       <c r="C12" t="str">
         <v>Invite to JRM</v>
@@ -644,18 +644,21 @@
         <v>FLCM</v>
       </c>
       <c r="E12" t="str">
-        <v>estimates</v>
+        <v>approved</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PDF</v>
       </c>
       <c r="G12">
-        <v>45700</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ENT-17089</v>
+        <v>ENT-17639</v>
       </c>
       <c r="B13" t="str">
-        <v>Cloudlink - LP1502 port</v>
+        <v>Send DAC ID to FIQM</v>
       </c>
       <c r="C13" t="str">
         <v>Invite to JRM</v>
@@ -667,15 +670,15 @@
         <v>estimates</v>
       </c>
       <c r="G13">
-        <v>45656</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ENT-16108</v>
+        <v>ENT-17089</v>
       </c>
       <c r="B14" t="str">
-        <v>Bring 2 workday views to our EDH Z4</v>
+        <v>Cloudlink - LP1502 port</v>
       </c>
       <c r="C14" t="str">
         <v>Invite to JRM</v>
@@ -687,15 +690,15 @@
         <v>estimates</v>
       </c>
       <c r="G14">
-        <v>45588</v>
+        <v>45656</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ENT-17559</v>
+        <v>ENT-16108</v>
       </c>
       <c r="B15" t="str">
-        <v>Data Source to EDGE</v>
+        <v>Bring 2 workday views to our EDH Z4</v>
       </c>
       <c r="C15" t="str">
         <v>Invite to JRM</v>
@@ -707,15 +710,15 @@
         <v>estimates</v>
       </c>
       <c r="G15">
-        <v>45664</v>
+        <v>45588</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ENT-17054</v>
+        <v>ENT-17559</v>
       </c>
       <c r="B16" t="str">
-        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
+        <v>Data Source to EDGE</v>
       </c>
       <c r="C16" t="str">
         <v>Invite to JRM</v>
@@ -724,21 +727,18 @@
         <v>FLCM</v>
       </c>
       <c r="E16" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F16" t="str">
-        <v>PDF</v>
+        <v>estimates</v>
       </c>
       <c r="G16">
-        <v>45691</v>
+        <v>45664</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">ENT-16009 </v>
+        <v>ENT-17054</v>
       </c>
       <c r="B17" t="str">
-        <v>Actimize Initiative - BSCM</v>
+        <v xml:space="preserve"> FLCM Case Type &amp; Records Modification</v>
       </c>
       <c r="C17" t="str">
         <v>Invite to JRM</v>
@@ -749,16 +749,19 @@
       <c r="E17" t="str">
         <v>approved</v>
       </c>
+      <c r="F17" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G17">
-        <v>45299</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ENT-14372</v>
+        <v xml:space="preserve">ENT-16009 </v>
       </c>
       <c r="B18" t="str">
-        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
+        <v>Actimize Initiative - BSCM</v>
       </c>
       <c r="C18" t="str">
         <v>Invite to JRM</v>
@@ -769,19 +772,16 @@
       <c r="E18" t="str">
         <v>approved</v>
       </c>
-      <c r="F18" t="str">
-        <v>PDF</v>
-      </c>
       <c r="G18">
-        <v>45512</v>
+        <v>45299</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ENT-16940</v>
+        <v>ENT-14372</v>
       </c>
       <c r="B19" t="str">
-        <v>RAMP Phase 2</v>
+        <v>Onboard Applications to TDE, DB Vault &amp; OKV</v>
       </c>
       <c r="C19" t="str">
         <v>Invite to JRM</v>
@@ -796,58 +796,58 @@
         <v>PDF</v>
       </c>
       <c r="G19">
-        <v>45562</v>
+        <v>45512</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>ENT-18473</v>
+        <v>ENT-16940</v>
       </c>
       <c r="B20" t="str">
-        <v xml:space="preserve">FCG Operating Model </v>
+        <v>RAMP Phase 2</v>
       </c>
       <c r="C20" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D20" t="str">
-        <v>FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E20" t="str">
-        <v>jrm</v>
+        <v>approved</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PDF</v>
       </c>
       <c r="G20">
-        <v>45695</v>
+        <v>45562</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ENT-17705</v>
+        <v>ENT-18473</v>
       </c>
       <c r="B21" t="str">
-        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
+        <v xml:space="preserve">FCG Operating Model </v>
       </c>
       <c r="C21" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D21" t="str">
-        <v>FLCM</v>
+        <v>FIQM</v>
       </c>
       <c r="E21" t="str">
-        <v>approved</v>
-      </c>
-      <c r="F21" t="str">
-        <v>PDF</v>
+        <v>jrm</v>
       </c>
       <c r="G21">
-        <v>45688</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>ENT-17213</v>
+        <v>ENT-17705</v>
       </c>
       <c r="B22" t="str">
-        <v>FLCM Upgrade and Enhancements ph2</v>
+        <v xml:space="preserve">eBit Web Service Migration Phase 2 </v>
       </c>
       <c r="C22" t="str">
         <v>Invite to JRM</v>
@@ -862,15 +862,15 @@
         <v>PDF</v>
       </c>
       <c r="G22">
-        <v>45701</v>
+        <v>45688</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ENT-17155</v>
+        <v>ENT-17213</v>
       </c>
       <c r="B23" t="str">
-        <v>NAE move to EDGE</v>
+        <v>FLCM Upgrade and Enhancements ph2</v>
       </c>
       <c r="C23" t="str">
         <v>Invite to JRM</v>
@@ -885,15 +885,15 @@
         <v>PDF</v>
       </c>
       <c r="G23">
-        <v>45695</v>
+        <v>45701</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>ENT-18591</v>
+        <v>ENT-17155</v>
       </c>
       <c r="B24" t="str">
-        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
+        <v>NAE move to EDGE</v>
       </c>
       <c r="C24" t="str">
         <v>Invite to JRM</v>
@@ -904,16 +904,19 @@
       <c r="E24" t="str">
         <v>approved</v>
       </c>
+      <c r="F24" t="str">
+        <v>PDF</v>
+      </c>
       <c r="G24">
-        <v>45706</v>
+        <v>45695</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>ENT-16938</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B25" t="str">
-        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
+        <v>FLCM - TII Data Governance - Work to Review Controls for Important and Core CDEs</v>
       </c>
       <c r="C25" t="str">
         <v>Invite to JRM</v>
@@ -922,138 +925,138 @@
         <v>FLCM</v>
       </c>
       <c r="E25" t="str">
-        <v>estimates</v>
+        <v>approved</v>
       </c>
       <c r="G25">
-        <v>45559</v>
+        <v>45706</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>ENT-17709</v>
+        <v>ENT-16938</v>
       </c>
       <c r="B26" t="str">
-        <v>CSDM Retention Policy Initiative</v>
+        <v>SAS Farm Data Exfiltration Risk Deficiency</v>
       </c>
       <c r="C26" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D26" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>FLCM</v>
       </c>
       <c r="E26" t="str">
         <v>estimates</v>
       </c>
       <c r="G26">
-        <v>45623</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ENT-13982</v>
+        <v>ENT-17709</v>
       </c>
       <c r="B27" t="str">
-        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
+        <v>CSDM Retention Policy Initiative</v>
       </c>
       <c r="C27" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D27" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E27" t="str">
         <v>estimates</v>
       </c>
       <c r="G27">
-        <v>45355</v>
+        <v>45623</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ENT-16173</v>
+        <v>ENT-13982</v>
       </c>
       <c r="B28" t="str">
-        <v>Move HR App off dedicated line</v>
+        <v>FINTRAC Incoming Cross Border e-Transfer Travel Rule (Reduced Scope – Reject Payments CBPT-2113)</v>
       </c>
       <c r="C28" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D28" t="str">
-        <v>CorpSec</v>
+        <v>FLCM</v>
       </c>
       <c r="E28" t="str">
         <v>estimates</v>
       </c>
       <c r="G28">
-        <v>45446</v>
+        <v>45355</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ENT-16787</v>
+        <v>ENT-16173</v>
       </c>
       <c r="B29" t="str">
-        <v>PES Historical Dart Report- Destruction</v>
+        <v>Move HR App off dedicated line</v>
       </c>
       <c r="C29" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D29" t="str">
-        <v>BSCM/ESCM</v>
+        <v>CorpSec</v>
       </c>
       <c r="E29" t="str">
         <v>estimates</v>
       </c>
       <c r="G29">
-        <v>45477</v>
+        <v>45446</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ENT-15671</v>
+        <v>ENT-16787</v>
       </c>
       <c r="B30" t="str">
-        <v>CSDM Upgrade</v>
+        <v>PES Historical Dart Report- Destruction</v>
       </c>
       <c r="C30" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D30" t="str">
-        <v>MinIO/DreamIO</v>
+        <v>BSCM/ESCM</v>
       </c>
       <c r="E30" t="str">
         <v>estimates</v>
       </c>
       <c r="G30">
-        <v>45394</v>
+        <v>45477</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>ENT-16956</v>
+        <v>ENT-15671</v>
       </c>
       <c r="B31" t="str">
-        <v>CPP - Consents and Enhanced Transparency - EDH</v>
+        <v>CSDM Upgrade</v>
       </c>
       <c r="C31" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D31" t="str">
-        <v>FLCM</v>
+        <v>MinIO/DreamIO</v>
       </c>
       <c r="E31" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G31">
-        <v>45531</v>
+        <v>45394</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>ENT-16024</v>
+        <v>ENT-16956</v>
       </c>
       <c r="B32" t="str">
-        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
+        <v>CPP - Consents and Enhanced Transparency - EDH</v>
       </c>
       <c r="C32" t="str">
         <v>Invite to JRM</v>
@@ -1065,15 +1068,15 @@
         <v>ofs</v>
       </c>
       <c r="G32">
-        <v>45453</v>
+        <v>45531</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>ENT-16511</v>
+        <v>ENT-16024</v>
       </c>
       <c r="B33" t="str">
-        <v>Horizon delta Migration | CIW Data Support</v>
+        <v>eBIT Migration Account Open Initiative: Estimates Request</v>
       </c>
       <c r="C33" t="str">
         <v>Invite to JRM</v>
@@ -1085,15 +1088,15 @@
         <v>ofs</v>
       </c>
       <c r="G33">
-        <v>45461</v>
+        <v>45453</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ENT-18723</v>
+        <v>ENT-16511</v>
       </c>
       <c r="B34" t="str">
-        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
+        <v>Horizon delta Migration | CIW Data Support</v>
       </c>
       <c r="C34" t="str">
         <v>Invite to JRM</v>
@@ -1102,95 +1105,98 @@
         <v>FLCM</v>
       </c>
       <c r="E34" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G34">
-        <v>45714</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>ENT-16748</v>
+        <v>ENT-18723</v>
       </c>
       <c r="B35" t="str">
-        <v>Project Mercury File Replacement</v>
+        <v>FLCM Account Table Update to Add New Suspense Accounts</v>
       </c>
       <c r="C35" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D35" t="str">
-        <v>FLCM/FIQM</v>
+        <v>FLCM</v>
       </c>
       <c r="E35" t="str">
-        <v>estimates</v>
+        <v>jrm</v>
       </c>
       <c r="G35">
-        <v>45686</v>
+        <v>45714</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ENT-15822</v>
+        <v>ENT-16748</v>
       </c>
       <c r="B36" t="str">
-        <v>CIPS - Fee Based Project</v>
+        <v>Project Mercury File Replacement</v>
       </c>
       <c r="C36" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D36" t="str">
-        <v>FLCM</v>
+        <v>FLCM/FIQM</v>
       </c>
       <c r="E36" t="str">
         <v>estimates</v>
       </c>
       <c r="G36">
-        <v>45650</v>
+        <v>45686</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v xml:space="preserve">ENT-16720 </v>
+        <v>ENT-15822</v>
       </c>
       <c r="B37" t="str">
-        <v>Corporate Security Data Management - POC request</v>
+        <v>CIPS - Fee Based Project</v>
       </c>
       <c r="C37" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="D37" t="str">
-        <v>BSCM/ESCM</v>
+        <v>FLCM</v>
       </c>
       <c r="E37" t="str">
         <v>estimates</v>
       </c>
       <c r="G37">
-        <v>45541</v>
+        <v>45650</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ENT-17853</v>
+        <v xml:space="preserve">ENT-16720 </v>
       </c>
       <c r="B38" t="str">
-        <v>ECIF R65 consumer regression testing</v>
+        <v>Corporate Security Data Management - POC request</v>
       </c>
       <c r="C38" t="str">
         <v>Invite to JRM</v>
       </c>
+      <c r="D38" t="str">
+        <v>BSCM/ESCM</v>
+      </c>
       <c r="E38" t="str">
-        <v>ofs</v>
+        <v>estimates</v>
       </c>
       <c r="G38">
-        <v>45691</v>
+        <v>45541</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>ENT-17109</v>
+        <v>ENT-17853</v>
       </c>
       <c r="B39" t="str">
-        <v>Mobile Credentials for Physical Access control</v>
+        <v>ECIF R65 consumer regression testing</v>
       </c>
       <c r="C39" t="str">
         <v>Invite to JRM</v>
@@ -1199,15 +1205,15 @@
         <v>ofs</v>
       </c>
       <c r="G39">
-        <v>45559</v>
+        <v>45691</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ENT-16786</v>
+        <v>ENT-17109</v>
       </c>
       <c r="B40" t="str">
-        <v>Fraud Mass Card Issuance</v>
+        <v>Mobile Credentials for Physical Access control</v>
       </c>
       <c r="C40" t="str">
         <v>Invite to JRM</v>
@@ -1216,15 +1222,15 @@
         <v>ofs</v>
       </c>
       <c r="G40">
-        <v>45596</v>
+        <v>45559</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>ENT-14160</v>
+        <v>ENT-16786</v>
       </c>
       <c r="B41" t="str">
-        <v>Create new NAE views and database roles</v>
+        <v>Fraud Mass Card Issuance</v>
       </c>
       <c r="C41" t="str">
         <v>Invite to JRM</v>
@@ -1233,15 +1239,15 @@
         <v>ofs</v>
       </c>
       <c r="G41">
-        <v>45378</v>
+        <v>45596</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>ENT-16394</v>
+        <v>ENT-14160</v>
       </c>
       <c r="B42" t="str">
-        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
+        <v>Create new NAE views and database roles</v>
       </c>
       <c r="C42" t="str">
         <v>Invite to JRM</v>
@@ -1250,15 +1256,15 @@
         <v>ofs</v>
       </c>
       <c r="G42">
-        <v>45468</v>
+        <v>45378</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>ENT-13691</v>
+        <v>ENT-16394</v>
       </c>
       <c r="B43" t="str">
-        <v>EAML Assurance &amp; FINTRAC Remediation</v>
+        <v>Visa Debit Int OCT - SLMS Adapter Update to Field 60</v>
       </c>
       <c r="C43" t="str">
         <v>Invite to JRM</v>
@@ -1267,15 +1273,15 @@
         <v>ofs</v>
       </c>
       <c r="G43">
-        <v>45310</v>
+        <v>45468</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>ENT-15815</v>
+        <v>ENT-13691</v>
       </c>
       <c r="B44" t="str">
-        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
+        <v>EAML Assurance &amp; FINTRAC Remediation</v>
       </c>
       <c r="C44" t="str">
         <v>Invite to JRM</v>
@@ -1284,15 +1290,15 @@
         <v>ofs</v>
       </c>
       <c r="G44">
-        <v>45427</v>
+        <v>45310</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>ENT-13593</v>
+        <v>ENT-15815</v>
       </c>
       <c r="B45" t="str">
-        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
+        <v>TSYS WCSA GL Keys Strategic Fix_PI3928</v>
       </c>
       <c r="C45" t="str">
         <v>Invite to JRM</v>
@@ -1301,15 +1307,15 @@
         <v>ofs</v>
       </c>
       <c r="G45">
-        <v>45279</v>
+        <v>45427</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>ENT-13829</v>
+        <v>ENT-13593</v>
       </c>
       <c r="B46" t="str">
-        <v>Quasi Cash - Modify MCC6540_PI3578</v>
+        <v>Bill C16 (Pronouns &amp; Clients Preferred Name)</v>
       </c>
       <c r="C46" t="str">
         <v>Invite to JRM</v>
@@ -1318,15 +1324,15 @@
         <v>ofs</v>
       </c>
       <c r="G46">
-        <v>45558</v>
+        <v>45279</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>ENT-14271</v>
+        <v>ENT-13829</v>
       </c>
       <c r="B47" t="str">
-        <v>EWM - OPF - Containerization - DEVO Integration</v>
+        <v>Quasi Cash - Modify MCC6540_PI3578</v>
       </c>
       <c r="C47" t="str">
         <v>Invite to JRM</v>
@@ -1335,15 +1341,15 @@
         <v>ofs</v>
       </c>
       <c r="G47">
-        <v>45383</v>
+        <v>45558</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>ENT-17801</v>
+        <v>ENT-14271</v>
       </c>
       <c r="B48" t="str">
-        <v>Avalor-Risk Orchestration POC</v>
+        <v>EWM - OPF - Containerization - DEVO Integration</v>
       </c>
       <c r="C48" t="str">
         <v>Invite to JRM</v>
@@ -1352,15 +1358,15 @@
         <v>ofs</v>
       </c>
       <c r="G48">
-        <v>45638</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>ENT-13880</v>
+        <v>ENT-17801</v>
       </c>
       <c r="B49" t="str">
-        <v>Artemis Program - Complaints Sustainment Improvements</v>
+        <v>Avalor-Risk Orchestration POC</v>
       </c>
       <c r="C49" t="str">
         <v>Invite to JRM</v>
@@ -1369,15 +1375,15 @@
         <v>ofs</v>
       </c>
       <c r="G49">
-        <v>45461</v>
+        <v>45638</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>ENT-14137</v>
+        <v>ENT-13880</v>
       </c>
       <c r="B50" t="str">
-        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
+        <v>Artemis Program - Complaints Sustainment Improvements</v>
       </c>
       <c r="C50" t="str">
         <v>Invite to JRM</v>
@@ -1386,15 +1392,15 @@
         <v>ofs</v>
       </c>
       <c r="G50">
-        <v>45371</v>
+        <v>45461</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ENT-14052</v>
+        <v>ENT-14137</v>
       </c>
       <c r="B51" t="str">
-        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
+        <v>Compass-AIM connectivity to allAccess for non-Core CIBC user info lookup</v>
       </c>
       <c r="C51" t="str">
         <v>Invite to JRM</v>
@@ -1408,10 +1414,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ENT-14203</v>
+        <v>ENT-14052</v>
       </c>
       <c r="B52" t="str">
-        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
+        <v>Costco Temp Cards Limit_PSBT-8200/DCTPI-3515</v>
       </c>
       <c r="C52" t="str">
         <v>Invite to JRM</v>
@@ -1420,15 +1426,15 @@
         <v>ofs</v>
       </c>
       <c r="G52">
-        <v>45406</v>
+        <v>45371</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ENT-14200</v>
+        <v>ENT-14203</v>
       </c>
       <c r="B53" t="str">
-        <v>WCSA GL Table Clean Up_PI3910</v>
+        <v>Bill C16 (Pronouns &amp; Client Preferred Name)</v>
       </c>
       <c r="C53" t="str">
         <v>Invite to JRM</v>
@@ -1437,15 +1443,15 @@
         <v>ofs</v>
       </c>
       <c r="G53">
-        <v>45364</v>
+        <v>45406</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ENT-13952</v>
+        <v>ENT-14200</v>
       </c>
       <c r="B54" t="str">
-        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
+        <v>WCSA GL Table Clean Up_PI3910</v>
       </c>
       <c r="C54" t="str">
         <v>Invite to JRM</v>
@@ -1454,15 +1460,15 @@
         <v>ofs</v>
       </c>
       <c r="G54">
-        <v>45593</v>
+        <v>45364</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ENT-15793</v>
+        <v>ENT-13952</v>
       </c>
       <c r="B55" t="str">
-        <v>Client Preference Center (CPC) - RBSS support</v>
+        <v>Credit Bureau Advancement 2.0 - Vulnerability Index</v>
       </c>
       <c r="C55" t="str">
         <v>Invite to JRM</v>
@@ -1471,15 +1477,15 @@
         <v>ofs</v>
       </c>
       <c r="G55">
-        <v>45408</v>
+        <v>45593</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ENT-16003</v>
+        <v>ENT-15793</v>
       </c>
       <c r="B56" t="str">
-        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
+        <v>Client Preference Center (CPC) - RBSS support</v>
       </c>
       <c r="C56" t="str">
         <v>Invite to JRM</v>
@@ -1488,15 +1494,15 @@
         <v>ofs</v>
       </c>
       <c r="G56">
-        <v>45595</v>
+        <v>45408</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ENT-15698</v>
+        <v>ENT-16003</v>
       </c>
       <c r="B57" t="str">
-        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
+        <v>Wires and Drafts Delegated and Supervisor Override Limits - RBSSINTK-9172</v>
       </c>
       <c r="C57" t="str">
         <v>Invite to JRM</v>
@@ -1505,15 +1511,15 @@
         <v>ofs</v>
       </c>
       <c r="G57">
-        <v>45392</v>
+        <v>45595</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ENT-15819</v>
+        <v>ENT-15698</v>
       </c>
       <c r="B58" t="str">
-        <v>Loan to Value (LTV)</v>
+        <v>Cards 21/5-day Offer Expiry Letters Process Enhancements</v>
       </c>
       <c r="C58" t="str">
         <v>Invite to JRM</v>
@@ -1522,15 +1528,15 @@
         <v>ofs</v>
       </c>
       <c r="G58">
-        <v>45411</v>
+        <v>45392</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>ENT-15919</v>
+        <v>ENT-15819</v>
       </c>
       <c r="B59" t="str">
-        <v>Business and Commercial Debit Card replacement</v>
+        <v>Loan to Value (LTV)</v>
       </c>
       <c r="C59" t="str">
         <v>Invite to JRM</v>
@@ -1544,27 +1550,27 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>ENT-18748</v>
+        <v>ENT-15919</v>
       </c>
       <c r="B60" t="str">
-        <v>CIP - PPS Readiness</v>
+        <v>Business and Commercial Debit Card replacement</v>
       </c>
       <c r="C60" t="str">
         <v>Invite to JRM</v>
       </c>
       <c r="E60" t="str">
-        <v>jrm</v>
+        <v>ofs</v>
       </c>
       <c r="G60">
-        <v>45721</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>ENT-18725</v>
+        <v>ENT-18748</v>
       </c>
       <c r="B61" t="str">
-        <v>US Video System - Lenel to Genetec</v>
+        <v>CIP - PPS Readiness</v>
       </c>
       <c r="C61" t="str">
         <v>Invite to JRM</v>
@@ -1576,9 +1582,26 @@
         <v>45721</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>ENT-18725</v>
+      </c>
+      <c r="B62" t="str">
+        <v>US Video System - Lenel to Genetec</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Invite to JRM</v>
+      </c>
+      <c r="E62" t="str">
+        <v>jrm</v>
+      </c>
+      <c r="G62">
+        <v>45721</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add new metrics data for 17054
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1548,7 +1548,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC8"/>
+  <dimension ref="A1:Z9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2157,10 +2157,89 @@
         <v>10</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>17054</v>
+      </c>
+      <c r="B9" t="str">
+        <v>344444</v>
+      </c>
+      <c r="C9" t="str">
+        <v>23424</v>
+      </c>
+      <c r="D9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="E9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="F9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="G9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="H9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="I9" t="str">
+        <v>24234</v>
+      </c>
+      <c r="J9" t="str">
+        <v>234</v>
+      </c>
+      <c r="K9" t="str">
+        <v>234</v>
+      </c>
+      <c r="L9" t="str">
+        <v>234</v>
+      </c>
+      <c r="M9" t="str">
+        <v>234</v>
+      </c>
+      <c r="N9" t="str">
+        <v>234</v>
+      </c>
+      <c r="O9" t="str">
+        <v>234</v>
+      </c>
+      <c r="P9" t="str">
+        <v>42</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="R9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="S9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="T9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="U9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="V9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="W9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="X9" t="str">
+        <v>234234</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>2342342</v>
+      </c>
+      <c r="Z9" t="str">
+        <v>342424</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new metrics data for 16009
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1615,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2304,9 +2304,89 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>16009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="C10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="D10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="E10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="F10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="G10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="H10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="I10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="J10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="K10" t="str">
+        <v>wer</v>
+      </c>
+      <c r="L10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="M10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="N10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="O10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="P10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="R10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="S10" t="str">
+        <v>234</v>
+      </c>
+      <c r="T10" t="str">
+        <v>234</v>
+      </c>
+      <c r="U10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="V10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="W10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="X10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>234234</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>234234</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new metrics data for ENT-18591
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1615,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2304,9 +2304,89 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ENT-18591</v>
+      </c>
+      <c r="B10" t="str">
+        <v>3434</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Delete Metrics row for ENT-16881
</commit_message>
<xml_diff>
--- a/Intake_Database.xlsx
+++ b/Intake_Database.xlsx
@@ -1615,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z10"/>
+  <dimension ref="A1:Z9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2226,10 +2226,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ENT-16881</v>
+        <v>ENT-18591</v>
       </c>
       <c r="B9" t="str">
-        <v>123123123</v>
+        <v>3434</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -2304,89 +2304,9 @@
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>ENT-18591</v>
-      </c>
-      <c r="B10" t="str">
-        <v>3434</v>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10" t="str">
-        <v/>
-      </c>
-      <c r="N10" t="str">
-        <v/>
-      </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
-        <v/>
-      </c>
-      <c r="R10" t="str">
-        <v/>
-      </c>
-      <c r="S10" t="str">
-        <v/>
-      </c>
-      <c r="T10" t="str">
-        <v/>
-      </c>
-      <c r="U10" t="str">
-        <v/>
-      </c>
-      <c r="V10" t="str">
-        <v/>
-      </c>
-      <c r="W10" t="str">
-        <v/>
-      </c>
-      <c r="X10" t="str">
-        <v/>
-      </c>
-      <c r="Y10" t="str">
-        <v/>
-      </c>
-      <c r="Z10" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>